<commit_message>
Correggi il file Excel che Excel segnalava come danneggiato
La cella con la formula di esempio nel foglio Soluzioni era salvata
come formula non valida: ora è testo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materiali/vendite_occhialeria_dolomiti.xlsx
+++ b/materiali/vendite_occhialeria_dolomiti.xlsx
@@ -4220,9 +4220,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13">
-        <f>SOMMA.SE(B2:B200; "Ottica Bianchi"; D2:D200)  → da usare nel foglio Vendite</f>
-        <v/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Formula (Excel in italiano): =SOMMA.SE(B2:B200; "Ottica Bianchi"; D2:D200) - da usare nel foglio Vendite</t>
+        </is>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Excel: una sola riga con la formula di controllo nel foglio Soluzioni
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materiali/vendite_occhialeria_dolomiti.xlsx
+++ b/materiali/vendite_occhialeria_dolomiti.xlsx
@@ -4069,7 +4069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4211,23 +4211,15 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Formula di controllo (Excel in italiano):</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Formula di controllo (Excel in italiano): =SOMMA.SE(B2:B200; "Ottica Bianchi"; D2:D200)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Formula (Excel in italiano): =SOMMA.SE(B2:B200; "Ottica Bianchi"; D2:D200) - da usare nel foglio Vendite</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Dati inventati a scopo didattico. Aziende e clienti non esistono.</t>
         </is>

</xml_diff>